<commit_message>
n8n board refresh 2026-07-15T17:39:53Z
</commit_message>
<xml_diff>
--- a/app/reports/GECC_research.xlsx
+++ b/app/reports/GECC_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-14 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-15 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>5.385</v>
+        <v>5.495</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04586999893188477</v>
+        <v>0.04549000263214111</v>
       </c>
     </row>
     <row r="6">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>13892045.31104921</v>
+        <v>13892044.40400364</v>
       </c>
     </row>
     <row r="36">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>5.385</v>
+        <v>5.495</v>
       </c>
     </row>
     <row r="38">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>74808664</v>
+        <v>76336784</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n"/>
@@ -1533,16 +1533,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>79458576</v>
+        <v>79735160</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>9.485849</v>
+        <v>9.518867999999999</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>4.099</v>
+        <v>4.065</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>1.415</v>
+        <v>1.403</v>
       </c>
     </row>
     <row r="8">
@@ -1557,14 +1557,14 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>6309846016</v>
+        <v>6831612928</v>
       </c>
       <c r="D8" s="33" t="n"/>
       <c r="E8" s="33" t="n">
-        <v>-64.51900000000001</v>
+        <v>-68.764</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>638.678</v>
+        <v>680.705</v>
       </c>
     </row>
     <row r="9">
@@ -1595,12 +1595,12 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>48099104</v>
+        <v>49036972</v>
       </c>
       <c r="D10" s="33" t="n"/>
       <c r="E10" s="33" t="n"/>
       <c r="F10" s="33" t="n">
-        <v>6.231</v>
+        <v>6.238</v>
       </c>
     </row>
     <row r="11">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C11" s="32" t="n"/>
       <c r="D11" s="33" t="n">
-        <v>16.22224</v>
+        <v>16.167612</v>
       </c>
       <c r="E11" s="33" t="n"/>
       <c r="F11" s="33" t="n"/>
@@ -1633,12 +1633,12 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>82753928</v>
+        <v>85034592</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n"/>
       <c r="F12" s="33" t="n">
-        <v>9.194000000000001</v>
+        <v>9.441000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1653,14 +1653,14 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>48989548</v>
+        <v>44935904</v>
       </c>
       <c r="D13" s="33" t="n"/>
       <c r="E13" s="33" t="n">
-        <v>-2.879</v>
+        <v>-2.799</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>-7.132</v>
+        <v>-6.934</v>
       </c>
     </row>
     <row r="15">

</xml_diff>